<commit_message>
Rework tables of functions and his counts
</commit_message>
<xml_diff>
--- a/compiler_practice_counts.xlsx
+++ b/compiler_practice_counts.xlsx
@@ -55,7 +55,7 @@
     <t xml:space="preserve">dead_code()</t>
   </si>
   <si>
-    <t xml:space="preserve">Одинаково</t>
+    <t xml:space="preserve">Clang / Intel</t>
   </si>
   <si>
     <t xml:space="preserve">unnecessary_loop()</t>
@@ -585,46 +585,46 @@
         <v>10</v>
       </c>
       <c r="B4" s="9" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4" s="9" t="n">
         <f aca="false">C4-B4</f>
-        <v>-8</v>
+        <v>-12</v>
       </c>
       <c r="E4" s="10" t="n">
         <f aca="false">D4/B4*100</f>
-        <v>-88.8888888888889</v>
+        <v>-70.5882352941177</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H4" s="9" t="n">
         <f aca="false">G4-F4</f>
-        <v>-7</v>
+        <v>-11</v>
       </c>
       <c r="I4" s="10" t="n">
         <f aca="false">H4/F4*100</f>
-        <v>-87.5</v>
+        <v>-78.5714285714286</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L4" s="9" t="n">
         <f aca="false">K4-J4</f>
-        <v>-7</v>
+        <v>-11</v>
       </c>
       <c r="M4" s="10" t="n">
         <f aca="false">L4/J4*100</f>
-        <v>-87.5</v>
+        <v>-78.5714285714286</v>
       </c>
       <c r="N4" s="11" t="s">
         <v>11</v>
@@ -635,49 +635,49 @@
         <v>12</v>
       </c>
       <c r="B5" s="9" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D5" s="9" t="n">
         <f aca="false">C5-B5</f>
-        <v>-19</v>
+        <v>-25</v>
       </c>
       <c r="E5" s="10" t="n">
         <f aca="false">D5/B5*100</f>
-        <v>-76</v>
+        <v>-71.4285714285714</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5" s="9" t="n">
         <f aca="false">G5-F5</f>
-        <v>-15</v>
+        <v>-22</v>
       </c>
       <c r="I5" s="10" t="n">
         <f aca="false">H5/F5*100</f>
-        <v>-71.4285714285714</v>
+        <v>-75.8620689655172</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L5" s="9" t="n">
         <f aca="false">K5-J5</f>
-        <v>-15</v>
+        <v>-19</v>
       </c>
       <c r="M5" s="10" t="n">
         <f aca="false">L5/J5*100</f>
-        <v>-71.4285714285714</v>
+        <v>-73.0769230769231</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -685,46 +685,46 @@
         <v>13</v>
       </c>
       <c r="B6" s="9" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">C6-B6</f>
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="E6" s="10" t="n">
         <f aca="false">D6/B6*100</f>
-        <v>-33.3333333333333</v>
+        <v>-25</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="H6" s="9" t="n">
         <f aca="false">G6-F6</f>
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I6" s="10" t="n">
         <f aca="false">H6/F6*100</f>
-        <v>-2.63157894736842</v>
+        <v>16.6666666666667</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="L6" s="9" t="n">
         <f aca="false">K6-J6</f>
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="M6" s="10" t="n">
         <f aca="false">L6/J6*100</f>
-        <v>60.5263157894737</v>
+        <v>95.2380952380952</v>
       </c>
       <c r="N6" s="11" t="s">
         <v>2</v>
@@ -735,10 +735,10 @@
         <v>14</v>
       </c>
       <c r="B7" s="9" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">C7-B7</f>
@@ -746,35 +746,35 @@
       </c>
       <c r="E7" s="10" t="n">
         <f aca="false">D7/B7*100</f>
-        <v>-43.75</v>
+        <v>-33.3333333333333</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="H7" s="9" t="n">
         <f aca="false">G7-F7</f>
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I7" s="10" t="n">
         <f aca="false">H7/F7*100</f>
-        <v>-4.34782608695652</v>
+        <v>17.8571428571429</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="L7" s="9" t="n">
         <f aca="false">K7-J7</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="M7" s="10" t="n">
         <f aca="false">L7/J7*100</f>
-        <v>42.8571428571429</v>
+        <v>53.8461538461539</v>
       </c>
       <c r="N7" s="11" t="s">
         <v>2</v>
@@ -785,46 +785,46 @@
         <v>15</v>
       </c>
       <c r="B8" s="9" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>43</v>
+        <v>78</v>
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">C8-B8</f>
-        <v>-7</v>
+        <v>13</v>
       </c>
       <c r="E8" s="10" t="n">
         <f aca="false">D8/B8*100</f>
-        <v>-14</v>
+        <v>20</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="H8" s="9" t="n">
         <f aca="false">G8-F8</f>
-        <v>-3</v>
+        <v>16</v>
       </c>
       <c r="I8" s="10" t="n">
         <f aca="false">H8/F8*100</f>
-        <v>-6</v>
+        <v>27.5862068965517</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="L8" s="9" t="n">
         <f aca="false">K8-J8</f>
-        <v>-10</v>
+        <v>2</v>
       </c>
       <c r="M8" s="10" t="n">
         <f aca="false">L8/J8*100</f>
-        <v>-20</v>
+        <v>3.44827586206897</v>
       </c>
       <c r="N8" s="11" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
Refresh counts of instructions
</commit_message>
<xml_diff>
--- a/compiler_practice_counts.xlsx
+++ b/compiler_practice_counts.xlsx
@@ -663,18 +663,18 @@
         <v>-75.8620689655172</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="K5" s="9" t="n">
         <v>7</v>
       </c>
       <c r="L5" s="9" t="n">
         <f aca="false">K5-J5</f>
-        <v>-19</v>
+        <v>-22</v>
       </c>
       <c r="M5" s="10" t="n">
         <f aca="false">L5/J5*100</f>
-        <v>-73.0769230769231</v>
+        <v>-75.8620689655172</v>
       </c>
       <c r="N5" s="11" t="s">
         <v>3</v>
@@ -699,32 +699,32 @@
         <v>-25</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H6" s="9" t="n">
         <f aca="false">G6-F6</f>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I6" s="10" t="n">
         <f aca="false">H6/F6*100</f>
-        <v>16.6666666666667</v>
+        <v>6.25</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>82</v>
       </c>
       <c r="L6" s="9" t="n">
         <f aca="false">K6-J6</f>
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="M6" s="10" t="n">
         <f aca="false">L6/J6*100</f>
-        <v>95.2380952380952</v>
+        <v>70.8333333333333</v>
       </c>
       <c r="N6" s="11" t="s">
         <v>2</v>
@@ -749,32 +749,32 @@
         <v>-33.3333333333333</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H7" s="9" t="n">
         <f aca="false">G7-F7</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I7" s="10" t="n">
         <f aca="false">H7/F7*100</f>
-        <v>17.8571428571429</v>
+        <v>9.67741935483871</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="K7" s="9" t="n">
         <v>40</v>
       </c>
       <c r="L7" s="9" t="n">
         <f aca="false">K7-J7</f>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="M7" s="10" t="n">
         <f aca="false">L7/J7*100</f>
-        <v>53.8461538461539</v>
+        <v>37.9310344827586</v>
       </c>
       <c r="N7" s="11" t="s">
         <v>2</v>
@@ -799,32 +799,32 @@
         <v>20</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H8" s="9" t="n">
         <f aca="false">G8-F8</f>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I8" s="10" t="n">
         <f aca="false">H8/F8*100</f>
-        <v>27.5862068965517</v>
+        <v>18.4615384615385</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L8" s="9" t="n">
         <f aca="false">K8-J8</f>
-        <v>2</v>
+        <v>-3</v>
       </c>
       <c r="M8" s="10" t="n">
         <f aca="false">L8/J8*100</f>
-        <v>3.44827586206897</v>
+        <v>-4.61538461538462</v>
       </c>
       <c r="N8" s="11" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
Add main function to analize. Update report to pattern
</commit_message>
<xml_diff>
--- a/compiler_practice_counts.xlsx
+++ b/compiler_practice_counts.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="17">
   <si>
     <t xml:space="preserve">Общее количество инструкций</t>
   </si>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t xml:space="preserve">jump_compression()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">main()</t>
   </si>
 </sst>
 </file>
@@ -663,18 +666,18 @@
         <v>-75.8620689655172</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K5" s="9" t="n">
         <v>7</v>
       </c>
       <c r="L5" s="9" t="n">
         <f aca="false">K5-J5</f>
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="M5" s="10" t="n">
         <f aca="false">L5/J5*100</f>
-        <v>-75.8620689655172</v>
+        <v>-75</v>
       </c>
       <c r="N5" s="11" t="s">
         <v>3</v>
@@ -699,32 +702,32 @@
         <v>-25</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G6" s="9" t="n">
         <v>51</v>
       </c>
       <c r="H6" s="9" t="n">
         <f aca="false">G6-F6</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" s="10" t="n">
         <f aca="false">H6/F6*100</f>
-        <v>6.25</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>82</v>
       </c>
       <c r="L6" s="9" t="n">
         <f aca="false">K6-J6</f>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M6" s="10" t="n">
         <f aca="false">L6/J6*100</f>
-        <v>70.8333333333333</v>
+        <v>78.2608695652174</v>
       </c>
       <c r="N6" s="11" t="s">
         <v>2</v>
@@ -763,18 +766,18 @@
         <v>9.67741935483871</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K7" s="9" t="n">
         <v>40</v>
       </c>
       <c r="L7" s="9" t="n">
         <f aca="false">K7-J7</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="M7" s="10" t="n">
         <f aca="false">L7/J7*100</f>
-        <v>37.9310344827586</v>
+        <v>48.1481481481481</v>
       </c>
       <c r="N7" s="11" t="s">
         <v>2</v>
@@ -802,32 +805,82 @@
         <v>65</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H8" s="9" t="n">
         <f aca="false">G8-F8</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I8" s="10" t="n">
         <f aca="false">H8/F8*100</f>
-        <v>18.4615384615385</v>
+        <v>16.9230769230769</v>
       </c>
       <c r="J8" s="9" t="n">
         <v>65</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L8" s="9" t="n">
         <f aca="false">K8-J8</f>
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="M8" s="10" t="n">
         <f aca="false">L8/J8*100</f>
-        <v>-4.61538461538462</v>
+        <v>-3.07692307692308</v>
       </c>
       <c r="N8" s="11" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>299</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <f aca="false">C9-B9</f>
+        <v>-131</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <f aca="false">D9/B9*100</f>
+        <v>-43.8127090301003</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>237</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>217</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <f aca="false">G9-F9</f>
+        <v>-20</v>
+      </c>
+      <c r="I9" s="10" t="n">
+        <f aca="false">H9/F9*100</f>
+        <v>-8.43881856540084</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>228</v>
+      </c>
+      <c r="K9" s="9" t="n">
+        <v>284</v>
+      </c>
+      <c r="L9" s="9" t="n">
+        <f aca="false">K9-J9</f>
+        <v>56</v>
+      </c>
+      <c r="M9" s="10" t="n">
+        <f aca="false">L9/J9*100</f>
+        <v>24.5614035087719</v>
+      </c>
+      <c r="N9" s="11" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>